<commit_message>
docs: sync design source tables and planning docs
</commit_message>
<xml_diff>
--- a/docs/product/design-source/蛋仔--大富翁--道具表.xlsx
+++ b/docs/product/design-source/蛋仔--大富翁--道具表.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\monopoly\design\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Administrator\Desktop\eggitor\1_开发中\大富翁\策划案\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C69B0A4-2038-4637-BDDF-07C96AF2B67C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931C87EB-CA69-4458-A59F-D50CB820526A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-930" yWindow="2055" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$2:$L$2</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -34,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="89">
   <si>
     <t>道具id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -56,10 +59,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>偷窃卡</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>怪兽卡</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -242,10 +241,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>使用导弹卡，你可以向前后3格范围内释放一枚导弹，摧毁该位置所有建筑、座驾，该位置玩家都住进医院。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>使用怪兽卡，你可以选择前后3格内的其他玩家建筑，释放怪兽拆除该建筑。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -370,10 +365,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>当你路过其他玩家时，你可以选择使用偷窃卡，获得他的一个道具。</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>有岔路机器人自动分裂，分别走多条路。</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -386,25 +377,19 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>offer_in_phases</t>
-  </si>
-  <si>
-    <t>post_action</t>
-  </si>
-  <si>
-    <t>pre_action</t>
-  </si>
-  <si>
-    <t>pre_move</t>
-  </si>
-  <si>
-    <t>pre_action,post_action</t>
-  </si>
-  <si>
-    <t>pass_player</t>
-  </si>
-  <si>
-    <t>tax_prompt</t>
+    <t>排序</t>
+  </si>
+  <si>
+    <t>使用窃取卡，选择一个有道具的玩家，窃取他的一个道具。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>窃取卡</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>选择一个其他玩家，向该玩家位置发射导弹，将该玩家送进医院，并摧毁该位置的建筑。</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -427,7 +412,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -443,6 +428,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B0F0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -474,11 +465,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -762,10 +754,10 @@
   <dimension ref="A1:L21"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="5" width="11.875" customWidth="1"/>
-    <col min="8" max="8" width="18.5" customWidth="1"/>
-    <col min="9" max="9" width="39.125" customWidth="1"/>
-    <col min="10" max="10" width="90" customWidth="1"/>
+    <col min="5" max="6" width="11.875" customWidth="1"/>
+    <col min="9" max="9" width="18.5" customWidth="1"/>
+    <col min="10" max="10" width="39.125" customWidth="1"/>
+    <col min="11" max="11" width="90" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12" x14ac:dyDescent="0.2">
@@ -773,37 +765,37 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>65</v>
+      <c r="D1" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>13</v>
+        <v>63</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>64</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>82</v>
+        <v>12</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>25</v>
-      </c>
       <c r="L1" s="2" t="s">
-        <v>88</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:12" x14ac:dyDescent="0.2">
@@ -811,25 +803,25 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="3" t="s">
         <v>1</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>81</v>
+        <v>1</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>4</v>
+        <v>79</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>4</v>
@@ -846,703 +838,708 @@
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
-        <v>2001</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E3" s="1">
-        <v>100</v>
+        <v>2003</v>
+      </c>
+      <c r="B3" s="2">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>65</v>
       </c>
       <c r="F3" s="1">
-        <v>500</v>
-      </c>
-      <c r="G3" s="1" t="b">
+        <v>5000</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1000</v>
+      </c>
+      <c r="H3" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H3" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="I3" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="J3" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="J3" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K3" s="1"/>
-      <c r="L3" s="1" t="s">
-        <v>89</v>
-      </c>
+      <c r="K3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L3" s="1"/>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2002</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="2">
+        <v>2</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F4" s="1">
+        <v>100</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1000</v>
+      </c>
+      <c r="H4" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="1">
-        <v>1</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E4" s="1">
-        <v>5000</v>
-      </c>
-      <c r="F4" s="1">
-        <v>1000</v>
-      </c>
-      <c r="G4" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="K4" s="1"/>
-      <c r="L4" s="1" t="s">
-        <v>90</v>
-      </c>
+      <c r="L4" s="1"/>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
-        <v>2003</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="1">
-        <v>1</v>
-      </c>
-      <c r="D5" s="1" t="s">
+        <v>2005</v>
+      </c>
+      <c r="B5" s="2">
+        <v>3</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
+      <c r="E5" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="E5" s="1">
-        <v>2500</v>
-      </c>
       <c r="F5" s="1">
+        <v>200</v>
+      </c>
+      <c r="G5" s="1">
         <v>1000</v>
       </c>
-      <c r="G5" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H5" s="1" t="s">
-        <v>30</v>
+      <c r="H5" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J5" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="K5" s="1"/>
+      <c r="K5" s="1" t="s">
+        <v>22</v>
+      </c>
       <c r="L5" s="1" t="s">
-        <v>91</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
-        <v>2004</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C6" s="1">
-        <v>1</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E6" s="1">
-        <v>5000</v>
+        <v>2012</v>
+      </c>
+      <c r="B6" s="2">
+        <v>4</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="1">
+        <v>1</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F6" s="1">
+        <v>5</v>
+      </c>
+      <c r="G6" s="1">
         <v>1000</v>
       </c>
-      <c r="G6" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" s="1" t="s">
-        <v>22</v>
+      <c r="H6" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="K6" s="1"/>
-      <c r="L6" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>50</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L6" s="1"/>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
-        <v>2005</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C7" s="1">
-        <v>1</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="1">
-        <v>2500</v>
+        <v>2004</v>
+      </c>
+      <c r="B7" s="2">
+        <v>5</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F7" s="1">
+        <v>5</v>
+      </c>
+      <c r="G7" s="1">
         <v>1000</v>
       </c>
-      <c r="G7" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>22</v>
+      <c r="H7" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>84</v>
+      </c>
+      <c r="L7" s="1"/>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>2006</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="2">
+        <v>6</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="1">
+        <v>5</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1000</v>
+      </c>
+      <c r="H8" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="1">
-        <v>1</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E8" s="1">
-        <v>2500</v>
-      </c>
-      <c r="F8" s="1">
-        <v>1000</v>
-      </c>
-      <c r="G8" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="I8" s="1" t="s">
+      <c r="K8" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="J8" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>85</v>
-      </c>
       <c r="L8" s="1" t="s">
-        <v>90</v>
+        <v>82</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
-        <v>2007</v>
-      </c>
-      <c r="B9" s="3" t="s">
+        <v>2001</v>
+      </c>
+      <c r="B9" s="2">
+        <v>7</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="1">
-        <v>2</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E9" s="1">
-        <v>100</v>
-      </c>
-      <c r="F9" s="1">
+      <c r="G9" s="1">
         <v>500</v>
       </c>
-      <c r="G9" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>24</v>
+      <c r="H9" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1" t="s">
-        <v>93</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L9" s="1"/>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
-        <v>2008</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" s="1">
+        <v>2007</v>
+      </c>
+      <c r="B10" s="2">
+        <v>8</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="1">
         <v>2</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="E10" s="1">
-        <v>100</v>
+      <c r="E10" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F10" s="1">
+        <v>10</v>
+      </c>
+      <c r="G10" s="1">
         <v>500</v>
       </c>
-      <c r="G10" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1" t="s">
-        <v>22</v>
+      <c r="H10" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="K10" s="1"/>
-      <c r="L10" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>35</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="L10" s="1"/>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
-        <v>2009</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C11" s="1">
+        <v>2008</v>
+      </c>
+      <c r="B11" s="2">
+        <v>9</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="1">
         <v>2</v>
       </c>
-      <c r="D11" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E11" s="1">
-        <v>5</v>
+      <c r="E11" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F11" s="1">
+        <v>10</v>
+      </c>
+      <c r="G11" s="1">
         <v>500</v>
       </c>
-      <c r="G11" s="1" t="b">
+      <c r="H11" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>19</v>
-      </c>
       <c r="I11" s="1" t="s">
-        <v>43</v>
+        <v>21</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>89</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="L11" s="1"/>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
-        <v>2010</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C12" s="1">
+        <v>2009</v>
+      </c>
+      <c r="B12" s="2">
+        <v>10</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="1">
         <v>2</v>
       </c>
-      <c r="D12" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E12" s="1">
-        <v>5</v>
+      <c r="E12" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F12" s="1">
-        <v>300</v>
-      </c>
-      <c r="G12" s="1" t="b">
+        <v>10</v>
+      </c>
+      <c r="G12" s="1">
+        <v>500</v>
+      </c>
+      <c r="H12" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="J12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="I12" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K12" s="1"/>
+      <c r="K12" s="1" t="s">
+        <v>39</v>
+      </c>
       <c r="L12" s="1" t="s">
-        <v>94</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
-        <v>2011</v>
-      </c>
-      <c r="B13" s="3" t="s">
+        <v>2013</v>
+      </c>
+      <c r="B13" s="2">
         <v>11</v>
       </c>
-      <c r="C13" s="1">
+      <c r="C13" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="1">
         <v>2</v>
       </c>
-      <c r="D13" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E13" s="1">
-        <v>50</v>
+      <c r="E13" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F13" s="1">
-        <v>50</v>
-      </c>
-      <c r="G13" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" s="1" t="s">
-        <v>22</v>
+        <v>10</v>
+      </c>
+      <c r="G13" s="1">
+        <v>500</v>
+      </c>
+      <c r="H13" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>50</v>
+        <v>21</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="K13" s="1"/>
+        <v>52</v>
+      </c>
+      <c r="K13" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="L13" s="1" t="s">
-        <v>92</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
-        <v>2012</v>
-      </c>
-      <c r="B14" s="3" t="s">
+        <v>2017</v>
+      </c>
+      <c r="B14" s="2">
         <v>12</v>
       </c>
-      <c r="C14" s="1">
-        <v>2</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="E14" s="1">
-        <v>5000</v>
+      <c r="C14" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="1">
+        <v>3</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F14" s="1">
-        <v>1000</v>
-      </c>
-      <c r="G14" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="G14" s="1">
+        <v>200</v>
+      </c>
+      <c r="H14" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>51</v>
+        <v>21</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="K14" s="1"/>
-      <c r="L14" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="L14" s="1"/>
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
-        <v>2013</v>
-      </c>
-      <c r="B15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C15" s="1">
+        <v>2018</v>
+      </c>
+      <c r="B15" s="2">
+        <v>13</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="D15" s="1">
         <v>3</v>
       </c>
-      <c r="D15" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E15" s="1">
-        <v>5</v>
+      <c r="E15" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F15" s="1">
-        <v>500</v>
-      </c>
-      <c r="G15" s="1" t="b">
+        <v>25</v>
+      </c>
+      <c r="G15" s="1">
+        <v>200</v>
+      </c>
+      <c r="H15" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H15" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="I15" s="1" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="L15" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>58</v>
+      </c>
+      <c r="L15" s="1"/>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
-        <v>2014</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>78</v>
-      </c>
-      <c r="C16" s="1">
+        <v>2019</v>
+      </c>
+      <c r="B16" s="2">
+        <v>14</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D16" s="1">
         <v>3</v>
       </c>
-      <c r="D16" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E16" s="1">
-        <v>50</v>
+      <c r="E16" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F16" s="1">
-        <v>150</v>
-      </c>
-      <c r="G16" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="G16" s="1">
+        <v>200</v>
+      </c>
+      <c r="H16" s="1" t="b">
+        <v>0</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>77</v>
+        <v>21</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>92</v>
+        <v>59</v>
       </c>
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
-        <v>2015</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="C17" s="1">
-        <v>3</v>
-      </c>
-      <c r="D17" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E17" s="1">
-        <v>20</v>
+        <v>2010</v>
+      </c>
+      <c r="B17" s="2">
+        <v>15</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="1">
+        <v>4</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F17" s="1">
-        <v>200</v>
-      </c>
-      <c r="G17" s="1" t="b">
+        <v>50</v>
+      </c>
+      <c r="G17" s="1">
+        <v>300</v>
+      </c>
+      <c r="H17" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="I17" s="1" t="s">
-        <v>70</v>
+        <v>41</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="K17" s="1"/>
-      <c r="L17" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>43</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="L17" s="1"/>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
-        <v>2016</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="C18" s="1">
-        <v>3</v>
-      </c>
-      <c r="D18" s="1" t="s">
+        <v>2015</v>
+      </c>
+      <c r="B18" s="2">
+        <v>16</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D18" s="1">
+        <v>4</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="F18" s="1">
+        <v>50</v>
+      </c>
+      <c r="G18" s="1">
+        <v>200</v>
+      </c>
+      <c r="H18" s="1" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="J18" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="E18" s="1">
-        <v>20</v>
-      </c>
-      <c r="F18" s="1">
-        <v>200</v>
-      </c>
-      <c r="G18" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H18" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="I18" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="J18" s="1" t="s">
-        <v>73</v>
-      </c>
       <c r="K18" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="L18" s="1" t="s">
-        <v>89</v>
-      </c>
+        <v>83</v>
+      </c>
+      <c r="L18" s="1"/>
     </row>
     <row r="19" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
-        <v>2017</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C19" s="1">
-        <v>3</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E19" s="1">
-        <v>10</v>
+        <v>2016</v>
+      </c>
+      <c r="B19" s="2">
+        <v>17</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D19" s="1">
+        <v>4</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F19" s="1">
+        <v>50</v>
+      </c>
+      <c r="G19" s="1">
         <v>200</v>
       </c>
-      <c r="G19" s="1" t="b">
+      <c r="H19" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>22</v>
-      </c>
       <c r="I19" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="K19" s="1"/>
+        <v>70</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>71</v>
+      </c>
       <c r="L19" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
-        <v>2018</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C20" s="1">
-        <v>3</v>
-      </c>
-      <c r="D20" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E20" s="1">
+        <v>2011</v>
+      </c>
+      <c r="B20" s="2">
+        <v>18</v>
+      </c>
+      <c r="C20" s="3" t="s">
         <v>10</v>
       </c>
+      <c r="D20" s="1">
+        <v>5</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>66</v>
+      </c>
       <c r="F20" s="1">
-        <v>200</v>
-      </c>
-      <c r="G20" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H20" s="1" t="s">
-        <v>22</v>
+        <v>100</v>
+      </c>
+      <c r="G20" s="1">
+        <v>50</v>
+      </c>
+      <c r="H20" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>62</v>
+        <v>21</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="K20" s="1"/>
-      <c r="L20" s="1" t="s">
-        <v>92</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="L20" s="1"/>
     </row>
     <row r="21" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
-        <v>2019</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="C21" s="1">
-        <v>3</v>
-      </c>
-      <c r="D21" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="E21" s="1">
-        <v>10</v>
+        <v>2014</v>
+      </c>
+      <c r="B21" s="2">
+        <v>19</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="D21" s="1">
+        <v>5</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>66</v>
       </c>
       <c r="F21" s="1">
-        <v>200</v>
-      </c>
-      <c r="G21" s="1" t="b">
-        <v>0</v>
-      </c>
-      <c r="H21" s="1" t="s">
-        <v>22</v>
+        <v>100</v>
+      </c>
+      <c r="G21" s="1">
+        <v>150</v>
+      </c>
+      <c r="H21" s="1" t="b">
+        <v>1</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>64</v>
+        <v>21</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>61</v>
+        <v>77</v>
       </c>
       <c r="L21" s="1" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A2:L2" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:L21">
+      <sortCondition ref="B2"/>
+    </sortState>
+  </autoFilter>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>